<commit_message>
feat: support 1 a 3 equipes, mode tinder 4 directions, purge auth_info et systeme de mise a jour
</commit_message>
<xml_diff>
--- a/Handball_Bot_Template.xlsx
+++ b/Handball_Bot_Template.xlsx
@@ -622,7 +622,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="B17:E22" displayName="Table_3" name="Table_3" id="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="B17:E29" displayName="Table_3" name="Table_3" id="3">
   <tableColumns count="4">
     <tableColumn name="Column1" id="1"/>
     <tableColumn name="Column2" id="2"/>
@@ -1071,6 +1071,132 @@
       <c r="D22" s="11"/>
       <c r="E22" s="11"/>
     </row>
+    <row r="23">
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Logo du Club (URL)</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>Lien direct vers l'image du blason</t>
+        </is>
+      </c>
+      <c r="E23" s="11"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Gymnase / Ville Domicile</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Gymnase Municipal</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>Nom de votre salle pour les matchs Ã  domicile</t>
+        </is>
+      </c>
+      <c r="E24" s="11"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>NumÃ©ros Coachs (ex: 336...)</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>33600000000</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>NumÃ©ros autorisÃ©s sÃ©parÃ©s par des virgules</t>
+        </is>
+      </c>
+      <c r="E25" s="11"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Couleur Principale Club (Hex)</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>#f97316</t>
+        </is>
+      </c>
+      <c r="D26" s="11" t="inlineStr">
+        <is>
+          <t>Couleur majeure (en-tÃªtes, boutons, accents)</t>
+        </is>
+      </c>
+      <c r="E26" s="11"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Couleur Secondaire Club (Hex)</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>#fbbf24</t>
+        </is>
+      </c>
+      <c r="D27" s="11" t="inlineStr">
+        <is>
+          <t>Couleur d'accent (dÃ©gradÃ©s, badges, notes)</t>
+        </is>
+      </c>
+      <c r="E27" s="11"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Couleur Ã‰quipe 1 (Hex)</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>#3b82f6</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="inlineStr">
+        <is>
+          <t>Couleur des maillots / colonne Ã‰quipe 1</t>
+        </is>
+      </c>
+      <c r="E28" s="11"/>
+    </row>
+    <row r="29">
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Couleur Ã‰quipe 2 (Hex)</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>#f97316</t>
+        </is>
+      </c>
+      <c r="D29" s="11" t="inlineStr">
+        <is>
+          <t>Couleur des maillots / colonne Ã‰quipe 2</t>
+        </is>
+      </c>
+      <c r="E29" s="11"/>
+    </row>
   </sheetData>
   <drawing r:id="rId3"/>
   <tableParts count="3">

</xml_diff>

<commit_message>
fix(xlsx): corriger l'encodage UTF-8 (mojibake) des chaines et en-tetes du template Excel
</commit_message>
<xml_diff>
--- a/Handball_Bot_Template.xlsx
+++ b/Handball_Bot_Template.xlsx
@@ -19,40 +19,40 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="80">
   <si>
-    <t>ParamÃ¨tres d'Automatisation - Handball Bot</t>
-  </si>
-  <si>
-    <t>Code Ã‰quipe</t>
-  </si>
-  <si>
-    <t>Nom recherchÃ© (Mot-clÃ© FFHB)</t>
-  </si>
-  <si>
-    <t>LibellÃ© dans le sondage</t>
-  </si>
-  <si>
-    <t>DÃ©lai RDV avant match (heures)</t>
+    <t>Paramètres d'Automatisation - Handball Bot</t>
+  </si>
+  <si>
+    <t>Code Équipe</t>
+  </si>
+  <si>
+    <t>Nom recherché (Mot-clé FFHB)</t>
+  </si>
+  <si>
+    <t>Libellé dans le sondage</t>
+  </si>
+  <si>
+    <t>Délai RDV avant match (heures)</t>
   </si>
   <si>
     <t>URL de la poule FFHB</t>
   </si>
   <si>
-    <t>Ã‰quipe 1</t>
+    <t>Équipe 1</t>
   </si>
   <si>
     <t>MON CLUB</t>
   </si>
   <si>
-    <t>Ã‰quipe 1</t>
+    <t>Équipe 1</t>
   </si>
   <si>
     <t>https://www.ffhandball.fr/competitions/...</t>
   </si>
   <si>
-    <t>Ã‰quipe 2</t>
-  </si>
-  <si>
-    <t>Ã‰quipe 2</t>
+    <t>Équipe 2</t>
+  </si>
+  <si>
+    <t>Équipe 2</t>
   </si>
   <si>
     <t>https://www.ffhandball.fr/competitions/...</t>
@@ -61,13 +61,13 @@
     <t>Ordre</t>
   </si>
   <si>
-    <t>IntitulÃ© de l'option dans le sondage</t>
+    <t>Intitulé de l'option dans le sondage</t>
   </si>
   <si>
     <t>Actif (OUI/NON)</t>
   </si>
   <si>
-    <t>EntraÃ®nement Lundi 20h30</t>
+    <t>Entraînement Lundi 20h30</t>
   </si>
   <si>
     <t>OUI</t>
@@ -76,19 +76,19 @@
     <t>ABS Lundi</t>
   </si>
   <si>
-    <t>EntraÃ®nement Mercredi 20h30</t>
+    <t>Entraînement Mercredi 20h30</t>
   </si>
   <si>
     <t>ABS Mercredi</t>
   </si>
   <si>
-    <t>EntraÃ®nement Jeudi 20h30</t>
+    <t>Entraînement Jeudi 20h30</t>
   </si>
   <si>
     <t>ABS Jeudi</t>
   </si>
   <si>
-    <t>ParamÃ¨tre</t>
+    <t>Paramètre</t>
   </si>
   <si>
     <t>Valeur</t>
@@ -106,7 +106,7 @@
     <t/>
   </si>
   <si>
-    <t>DÃ©pÃ´t GitHub (owner/repo)</t>
+    <t>Dépôt GitHub (owner/repo)</t>
   </si>
   <si>
     <t>votre-pseudo/handball-bot</t>
@@ -133,7 +133,7 @@
     <t>Date validation</t>
   </si>
   <si>
-    <t>SÃ©ance</t>
+    <t>Séance</t>
   </si>
   <si>
     <t>Groupe 1 / Effectif retenu</t>
@@ -148,13 +148,13 @@
     <t>Nom / Surnom</t>
   </si>
   <si>
-    <t>TÃ©lÃ©phone (format 336...)</t>
+    <t>Téléphone (format 336...)</t>
   </si>
   <si>
     <t>Poste</t>
   </si>
   <si>
-    <t>Ã‰quipe habituelle</t>
+    <t>Équipe habituelle</t>
   </si>
   <si>
     <t>Photo (URL ou lien Drive)</t>
@@ -193,13 +193,13 @@
     <t>Alexandre Petit</t>
   </si>
   <si>
-    <t>ArriÃ¨re Droit</t>
+    <t>Arrière Droit</t>
   </si>
   <si>
     <t>Romain Laurent</t>
   </si>
   <si>
-    <t>ArriÃ¨re Gauche</t>
+    <t>Arrière Gauche</t>
   </si>
   <si>
     <t>Capitaine</t>
@@ -208,13 +208,13 @@
     <t>Joueur</t>
   </si>
   <si>
-    <t>Nb EntraÃ®nements (0-3)</t>
-  </si>
-  <si>
-    <t>Dispo Ã‰quipe 1</t>
-  </si>
-  <si>
-    <t>Dispo Ã‰quipe 2</t>
+    <t>Nb Entraînements (0-3)</t>
+  </si>
+  <si>
+    <t>Dispo Équipe 1</t>
+  </si>
+  <si>
+    <t>Dispo Équipe 2</t>
   </si>
   <si>
     <t>Dispo Lundi</t>
@@ -226,13 +226,13 @@
     <t>Dispo Jeudi</t>
   </si>
   <si>
-    <t>Non convoquÃ©s</t>
-  </si>
-  <si>
-    <t>Matchs DÃ©tectÃ©s par le Script (Exemple)</t>
-  </si>
-  <si>
-    <t>AperÃ§u du prochain sondage WhatsApp</t>
+    <t>Non convoqués</t>
+  </si>
+  <si>
+    <t>Matchs Détectés par le Script (Exemple)</t>
+  </si>
+  <si>
+    <t>Aperçu du prochain sondage WhatsApp</t>
   </si>
   <si>
     <t>Choix multiples : OUI (selectableCount = 0)</t>
@@ -253,7 +253,7 @@
     <t>Heure RDV</t>
   </si>
   <si>
-    <t>Lieu (Domicile / ExtÃ©rieur)</t>
+    <t>Lieu (Domicile / Extérieur)</t>
   </si>
   <si>
     <t>Adversaire</t>
@@ -622,7 +622,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="B17:E29" displayName="Table_3" name="Table_3" id="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="B17:E22" displayName="Table_3" name="Table_3" id="3">
   <tableColumns count="4">
     <tableColumn name="Column1" id="1"/>
     <tableColumn name="Column2" id="2"/>
@@ -1071,132 +1071,6 @@
       <c r="D22" s="11"/>
       <c r="E22" s="11"/>
     </row>
-    <row r="23">
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>Logo du Club (URL)</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="D23" s="11" t="inlineStr">
-        <is>
-          <t>Lien direct vers l'image du blason</t>
-        </is>
-      </c>
-      <c r="E23" s="11"/>
-    </row>
-    <row r="24">
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>Gymnase / Ville Domicile</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>Gymnase Municipal</t>
-        </is>
-      </c>
-      <c r="D24" s="11" t="inlineStr">
-        <is>
-          <t>Nom de votre salle pour les matchs Ã  domicile</t>
-        </is>
-      </c>
-      <c r="E24" s="11"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>NumÃ©ros Coachs (ex: 336...)</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>33600000000</t>
-        </is>
-      </c>
-      <c r="D25" s="11" t="inlineStr">
-        <is>
-          <t>NumÃ©ros autorisÃ©s sÃ©parÃ©s par des virgules</t>
-        </is>
-      </c>
-      <c r="E25" s="11"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>Couleur Principale Club (Hex)</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>#f97316</t>
-        </is>
-      </c>
-      <c r="D26" s="11" t="inlineStr">
-        <is>
-          <t>Couleur majeure (en-tÃªtes, boutons, accents)</t>
-        </is>
-      </c>
-      <c r="E26" s="11"/>
-    </row>
-    <row r="27">
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>Couleur Secondaire Club (Hex)</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>#fbbf24</t>
-        </is>
-      </c>
-      <c r="D27" s="11" t="inlineStr">
-        <is>
-          <t>Couleur d'accent (dÃ©gradÃ©s, badges, notes)</t>
-        </is>
-      </c>
-      <c r="E27" s="11"/>
-    </row>
-    <row r="28">
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>Couleur Ã‰quipe 1 (Hex)</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>#3b82f6</t>
-        </is>
-      </c>
-      <c r="D28" s="11" t="inlineStr">
-        <is>
-          <t>Couleur des maillots / colonne Ã‰quipe 1</t>
-        </is>
-      </c>
-      <c r="E28" s="11"/>
-    </row>
-    <row r="29">
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>Couleur Ã‰quipe 2 (Hex)</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>#f97316</t>
-        </is>
-      </c>
-      <c r="D29" s="11" t="inlineStr">
-        <is>
-          <t>Couleur des maillots / colonne Ã‰quipe 2</t>
-        </is>
-      </c>
-      <c r="E29" s="11"/>
-    </row>
   </sheetData>
   <drawing r:id="rId3"/>
   <tableParts count="3">

</xml_diff>

<commit_message>
feat(template): integrer par defaut les 3 equipes pretes dans le tableau et initialisation
</commit_message>
<xml_diff>
--- a/Handball_Bot_Template.xlsx
+++ b/Handball_Bot_Template.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="82">
   <si>
     <t>Paramètres d'Automatisation - Handball Bot</t>
   </si>
@@ -257,6 +257,12 @@
   </si>
   <si>
     <t>Adversaire</t>
+  </si>
+  <si>
+    <t>Équipe 3</t>
+  </si>
+  <si>
+    <t>Dispo Équipe 3</t>
   </si>
 </sst>
 </file>
@@ -598,7 +604,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="B3:F5" displayName="Table_1" name="Table_1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="B3:F6" displayName="Table_1" name="Table_1" id="1">
   <tableColumns count="5">
     <tableColumn name="Code Équipe" id="1"/>
     <tableColumn name="Nom recherché (Mot-clé FFHB)" id="2"/>
@@ -930,6 +936,23 @@
         <v>12</v>
       </c>
     </row>
+    <row r="6">
+      <c r="B6" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="E6" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
     <row r="8">
       <c r="B8" s="2" t="s">
         <v>13</v>
@@ -1256,12 +1279,15 @@
         <v>65</v>
       </c>
       <c r="F1" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="G1" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="G1" s="14" t="s">
+      <c r="H1" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="H1" s="14" t="s">
+      <c r="I1" s="14" t="s">
         <v>68</v>
       </c>
     </row>
@@ -1279,7 +1305,9 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="14.0"/>
     <col customWidth="1" min="2" max="2" width="25.25"/>
-    <col customWidth="1" min="3" max="3" width="41.88"/>
+    <col customWidth="1" min="3" max="3" width="25.25"/>
+    <col customWidth="1" min="4" max="4" width="25.25"/>
+    <col customWidth="1" min="5" max="5" width="41.88"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1293,6 +1321,9 @@
         <v>11</v>
       </c>
       <c r="D1" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="E1" s="14" t="s">
         <v>69</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(config): selection du nombre d'equipes (1, 2 ou 3) a l'initialisation et 3 par defaut dans le template
</commit_message>
<xml_diff>
--- a/Handball_Bot_Template.xlsx
+++ b/Handball_Bot_Template.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="107">
   <si>
     <t>Paramètres d'Automatisation - Handball Bot</t>
   </si>
@@ -103,7 +103,8 @@
     <t>120363xxxxxxxxx@g.us</t>
   </si>
   <si>
-    <t/>
+    <t>
+    </t>
   </si>
   <si>
     <t>Dépôt GitHub (owner/repo)</t>
@@ -121,7 +122,8 @@
     <t>URL WebApp (Auto)</t>
   </si>
   <si>
-    <t/>
+    <t>
+    </t>
   </si>
   <si>
     <t>Nom du Club</t>
@@ -263,6 +265,81 @@
   </si>
   <si>
     <t>Dispo Équipe 3</t>
+  </si>
+  <si>
+    <t>Logo du Club (URL)</t>
+  </si>
+  <si>
+    <t>Lien direct vers le blason (ou vide pour logo auto)</t>
+  </si>
+  <si>
+    <t>Gymnase / Ville Domicile</t>
+  </si>
+  <si>
+    <t>Gymnase Municipal</t>
+  </si>
+  <si>
+    <t>Nom de votre salle pour les matchs à domicile</t>
+  </si>
+  <si>
+    <t>Numéros Coachs (ex: 336...)</t>
+  </si>
+  <si>
+    <t>33600000000</t>
+  </si>
+  <si>
+    <t>Numéros des coachs autorisés (séparés par virgules)</t>
+  </si>
+  <si>
+    <t>Couleur Principale Club (Hex)</t>
+  </si>
+  <si>
+    <t>#f97316</t>
+  </si>
+  <si>
+    <t>Aperçu</t>
+  </si>
+  <si>
+    <t>Couleur majeure (en-têtes, boutons, accents)</t>
+  </si>
+  <si>
+    <t>Couleur Secondaire Club (Hex)</t>
+  </si>
+  <si>
+    <t>#fbbf24</t>
+  </si>
+  <si>
+    <t>Couleur d'accent (dégradés, badges, notes)</t>
+  </si>
+  <si>
+    <t>Couleur Équipe 1 (Hex)</t>
+  </si>
+  <si>
+    <t>#3b82f6</t>
+  </si>
+  <si>
+    <t>Couleur des maillots / colonne Équipe 1</t>
+  </si>
+  <si>
+    <t>Couleur Équipe 2 (Hex)</t>
+  </si>
+  <si>
+    <t>Couleur des maillots / colonne Équipe 2</t>
+  </si>
+  <si>
+    <t>Couleur Équipe 3 (Hex)</t>
+  </si>
+  <si>
+    <t>#10b981</t>
+  </si>
+  <si>
+    <t>Couleur des maillots / colonne Équipe 3</t>
+  </si>
+  <si>
+    <t>Nombre d'Équipes dans le groupe</t>
+  </si>
+  <si>
+    <t>Nombre d'équipes gérées (1, 2 ou 3 - défaut : 3)</t>
   </si>
 </sst>
 </file>
@@ -628,7 +705,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="B17:E22" displayName="Table_3" name="Table_3" id="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="B17:E31" displayName="Table_3" name="Table_3" id="3">
   <tableColumns count="4">
     <tableColumn name="Column1" id="1"/>
     <tableColumn name="Column2" id="2"/>
@@ -1094,6 +1171,124 @@
       <c r="D22" s="11"/>
       <c r="E22" s="11"/>
     </row>
+    <row r="23">
+      <c r="B23" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D23" s="6"/>
+      <c r="E23" s="7" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D24" s="6"/>
+      <c r="E24" s="7" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D25" s="6"/>
+      <c r="E25" s="7" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="E26" s="7" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="E27" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="E28" s="7" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="E29" s="7" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="E30" s="7" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C31" s="3">
+        <v>3</v>
+      </c>
+      <c r="D31" s="6"/>
+      <c r="E31" s="7" t="s">
+        <v>106</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId3"/>
   <tableParts count="3">

</xml_diff>

<commit_message>
feat(template): mise a jour complete du fichier Handball_Bot_Template.xlsx et alignement avec le code
</commit_message>
<xml_diff>
--- a/Handball_Bot_Template.xlsx
+++ b/Handball_Bot_Template.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="113">
   <si>
     <t>Paramètres d'Automatisation - Handball Bot</t>
   </si>
@@ -340,6 +340,24 @@
   </si>
   <si>
     <t>Nombre d'équipes gérées (1, 2 ou 3 - défaut : 3)</t>
+  </si>
+  <si>
+    <t>Page FFHB du Club (URL)</t>
+  </si>
+  <si>
+    <t>Lien vers monclub.ffhandball.fr (logo et couleurs auto)</t>
+  </si>
+  <si>
+    <t>Salle / Gymnase</t>
+  </si>
+  <si>
+    <t>Option générée pour WhatsApp</t>
+  </si>
+  <si>
+    <t>Statut</t>
+  </si>
+  <si>
+    <t>Équipe</t>
   </si>
 </sst>
 </file>
@@ -705,7 +723,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="B17:E31" displayName="Table_3" name="Table_3" id="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="B17:E32" displayName="Table_3" name="Table_3" id="3">
   <tableColumns count="4">
     <tableColumn name="Column1" id="1"/>
     <tableColumn name="Column2" id="2"/>
@@ -1289,6 +1307,18 @@
         <v>106</v>
       </c>
     </row>
+    <row r="32">
+      <c r="B32" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D32" s="6"/>
+      <c r="E32" s="7" t="s">
+        <v>108</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId3"/>
   <tableParts count="3">
@@ -1556,7 +1586,7 @@
         <v>74</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>1</v>
+        <v>112</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>75</v>
@@ -1574,13 +1604,13 @@
         <v>79</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>44</v>
+        <v>109</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>14</v>
+        <v>110</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>23</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>